<commit_message>
docs(custos): adiciona voz (ElevenLabs TTS + Deepgram STT) à unit economics
Novas linhas na aba Custos: TTS (ElevenLabs Turbo v2.5, US$0,05/1k chars) e
STT (Deepgram Nova-3, US$0,0077/min streaming). Total de IA agora soma voz e
o Resumo referencia as novas linhas.

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Maya_Unit_Economics.xlsx
+++ b/Maya_Unit_Economics.xlsx
@@ -199,7 +199,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -244,6 +244,10 @@
     <xf numFmtId="9" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="9" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -719,7 +723,7 @@
         </is>
       </c>
       <c r="B12" s="6">
-        <f>Custos!B21</f>
+        <f>Custos!B22</f>
         <v/>
       </c>
     </row>
@@ -730,7 +734,7 @@
         </is>
       </c>
       <c r="B13" s="6">
-        <f>Custos!B22</f>
+        <f>Custos!B23</f>
         <v/>
       </c>
     </row>
@@ -987,7 +991,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="46.109375" bestFit="1" customWidth="1" style="17" min="1" max="1"/>
@@ -1007,7 +1011,7 @@
     <row r="2">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Modelos: Haiku 4.5 = $1/M in / $5/M out  •  Sonnet 5 = $3/M in / $15/M out (tarifa padrão, após 31/08/2026).</t>
+          <t>Modelos: Haiku 4.5 = $1/M in / $5/M out  •  Sonnet 5 = $3/M in / $15/M out (tarifa padrão, após 31/08/2026).  •  Voz: ElevenLabs Turbo v2.5 = US$0,05/1k chars  •  Deepgram Nova-3 = US$0,0077/min (streaming).</t>
         </is>
       </c>
     </row>
@@ -1404,50 +1408,105 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>TTS — voz da Maya</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ElevenLabs Turbo v2.5</t>
+        </is>
+      </c>
+      <c r="C20" s="38" t="n">
+        <v>400</v>
+      </c>
+      <c r="E20" s="39" t="n">
+        <v>40</v>
+      </c>
+      <c r="F20" s="40">
+        <f>E20*C20/1000*0.05</f>
+        <v/>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>US$0,05/1k chars; ~400 chars/resposta</t>
+        </is>
+      </c>
+    </row>
     <row r="21">
-      <c r="A21" s="14" t="inlineStr">
-        <is>
-          <t>TOTAL LLM / usuário / mês (USD)</t>
-        </is>
-      </c>
-      <c r="B21" s="12">
-        <f>SUM(F10:F19)</f>
-        <v/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>STT — transcrição de voz</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Deepgram Nova-3</t>
+        </is>
+      </c>
+      <c r="C21" s="38" t="n">
+        <v>15</v>
+      </c>
+      <c r="E21" s="39" t="n">
+        <v>40</v>
+      </c>
+      <c r="F21" s="40">
+        <f>E21*C21/60*0.0077</f>
+        <v/>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>US$0,0077/min (streaming); ~15s/áudio</t>
+        </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>TOTAL IA (LLM + voz) / usuário / mês (USD)</t>
+        </is>
+      </c>
+      <c r="B22" s="41">
+        <f>SUM(F10:F21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
         <is>
           <t>Infra fixa (Supabase/Vercel/Mapbox/push) / mês (USD)</t>
         </is>
       </c>
-      <c r="B22" s="2" t="n">
+      <c r="B23" s="2" t="n">
         <v>0.1</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="14" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <t>COGS TOTAL / usuário / mês (USD)</t>
         </is>
       </c>
-      <c r="B23" s="12">
-        <f>B21+B22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="20" t="inlineStr">
-        <is>
-          <t>Cenários (edite a coluna 'Chamadas/mês'): usuário casual ~US$0,50-1,50  •  médio ~US$2-3  •  power user ~US$5-8.</t>
-        </is>
-      </c>
-      <c r="B25" s="21" t="n"/>
-      <c r="C25" s="21" t="n"/>
-      <c r="D25" s="21" t="n"/>
-      <c r="E25" s="21" t="n"/>
-      <c r="F25" s="21" t="n"/>
-      <c r="G25" s="22" t="n"/>
+      <c r="B24" s="41">
+        <f>B22+B23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
+          <t>Cenários (edite a coluna 'Chamadas/mês'): usuário casual ~US$0,50-1,50  •  médio ~US$2-3  •  power user ~US$5-8  •  voz adiciona ~US$0,50-1,00 (médio).</t>
+        </is>
+      </c>
+      <c r="B26" s="21" t="n"/>
+      <c r="C26" s="21" t="n"/>
+      <c r="D26" s="21" t="n"/>
+      <c r="E26" s="21" t="n"/>
+      <c r="F26" s="21" t="n"/>
+      <c r="G26" s="22" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>